<commit_message>
Enforce highest win percentage gate, fix unsettled picks, promote CFB v2, restructure sports directory
</commit_message>
<xml_diff>
--- a/data/sports/dota2/gated.xlsx
+++ b/data/sports/dota2/gated.xlsx
@@ -300,8 +300,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="PicksLedger" displayName="PicksLedger" ref="A1:DQ116" headerRowCount="1">
-  <autoFilter ref="A1:DQ116"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="PicksLedger" displayName="PicksLedger" ref="A1:DQ119" headerRowCount="1">
+  <autoFilter ref="A1:DQ119"/>
   <tableColumns count="121">
     <tableColumn id="1" name="pick_id"/>
     <tableColumn id="2" name="created_at_utc"/>
@@ -780,19 +780,19 @@
     </row>
     <row r="4" ht="28" customHeight="1">
       <c r="A4" s="6">
-        <f>COUNTA('Picks'!$A$2:$A$116)</f>
+        <f>COUNTA('Picks'!$A$2:$A$119)</f>
         <v/>
       </c>
       <c r="C4" s="6">
-        <f>COUNTIF('Picks'!$U$2:$U$116,"open")</f>
+        <f>COUNTIF('Picks'!$U$2:$U$119,"open")</f>
         <v/>
       </c>
       <c r="E4" s="6">
-        <f>COUNTIF('Picks'!$U$2:$U$116,"settled")</f>
+        <f>COUNTIF('Picks'!$U$2:$U$119,"settled")</f>
         <v/>
       </c>
       <c r="G4" s="6">
-        <f>IF(COUNTIFS('Picks'!$U$2:$U$116,"settled",'Picks'!$V$2:$V$116,"win")+COUNTIFS('Picks'!$U$2:$U$116,"settled",'Picks'!$V$2:$V$116,"loss")&gt;=$L$2,"Ready","Insufficient sample")</f>
+        <f>IF(COUNTIFS('Picks'!$U$2:$U$119,"settled",'Picks'!$V$2:$V$119,"win")+COUNTIFS('Picks'!$U$2:$U$119,"settled",'Picks'!$V$2:$V$119,"loss")&gt;=$L$2,"Ready","Insufficient sample")</f>
         <v/>
       </c>
     </row>
@@ -820,19 +820,19 @@
     </row>
     <row r="7" ht="28" customHeight="1">
       <c r="A7" s="6">
-        <f>COUNTIF('Picks'!$BX$2:$BX$116,"&gt;0")</f>
+        <f>COUNTIF('Picks'!$BX$2:$BX$119,"&gt;0")</f>
         <v/>
       </c>
       <c r="C7" s="6">
-        <f>COUNTIFS('Picks'!$BX$2:$BX$116,"&gt;0",'Picks'!$V$2:$V$116,"win")&amp;"-"&amp;COUNTIFS('Picks'!$BX$2:$BX$116,"&gt;0",'Picks'!$V$2:$V$116,"loss")</f>
+        <f>COUNTIFS('Picks'!$BX$2:$BX$119,"&gt;0",'Picks'!$V$2:$V$119,"win")&amp;"-"&amp;COUNTIFS('Picks'!$BX$2:$BX$119,"&gt;0",'Picks'!$V$2:$V$119,"loss")</f>
         <v/>
       </c>
       <c r="E7" s="7">
-        <f>IFERROR(COUNTIFS('Picks'!$BX$2:$BX$116,"&gt;0",'Picks'!$V$2:$V$116,"win")/(COUNTIFS('Picks'!$BX$2:$BX$116,"&gt;0",'Picks'!$V$2:$V$116,"win")+COUNTIFS('Picks'!$BX$2:$BX$116,"&gt;0",'Picks'!$V$2:$V$116,"loss")),0)</f>
+        <f>IFERROR(COUNTIFS('Picks'!$BX$2:$BX$119,"&gt;0",'Picks'!$V$2:$V$119,"win")/(COUNTIFS('Picks'!$BX$2:$BX$119,"&gt;0",'Picks'!$V$2:$V$119,"win")+COUNTIFS('Picks'!$BX$2:$BX$119,"&gt;0",'Picks'!$V$2:$V$119,"loss")),0)</f>
         <v/>
       </c>
       <c r="G7" s="7">
-        <f>IFERROR(SUM('Picks'!$BY$2:$BY$116)/SUM('Picks'!$BX$2:$BX$116),0)</f>
+        <f>IFERROR(SUM('Picks'!$BY$2:$BY$119)/SUM('Picks'!$BX$2:$BX$119),0)</f>
         <v/>
       </c>
     </row>
@@ -860,19 +860,19 @@
     </row>
     <row r="10" ht="28" customHeight="1">
       <c r="A10" s="8">
-        <f>SUM('Picks'!$BY$2:$BY$116)</f>
+        <f>SUM('Picks'!$BY$2:$BY$119)</f>
         <v/>
       </c>
       <c r="C10" s="9">
-        <f>IFERROR(AVERAGEIF('Picks'!$AB$2:$AB$116,"&lt;&gt;",'Picks'!$AB$2:$AB$116),0)</f>
+        <f>IFERROR(AVERAGEIF('Picks'!$AB$2:$AB$119,"&lt;&gt;",'Picks'!$AB$2:$AB$119),0)</f>
         <v/>
       </c>
       <c r="E10" s="6">
-        <f>COUNTIFS('Picks'!$AM$2:$AM$116,"QUALIFIED_SHADOW_CALL",'Picks'!$U$2:$U$116,"settled")</f>
+        <f>COUNTIFS('Picks'!$AM$2:$AM$119,"QUALIFIED_SHADOW_CALL",'Picks'!$U$2:$U$119,"settled")</f>
         <v/>
       </c>
       <c r="G10" s="8">
-        <f>SUMIFS('Picks'!$AC$2:$AC$116,'Picks'!$AM$2:$AM$116,"QUALIFIED_SHADOW_CALL")</f>
+        <f>SUMIFS('Picks'!$AC$2:$AC$119,'Picks'!$AM$2:$AM$119,"QUALIFIED_SHADOW_CALL")</f>
         <v/>
       </c>
     </row>
@@ -927,15 +927,15 @@
         </is>
       </c>
       <c r="B14" s="13">
-        <f>COUNTIFS('Picks'!$H$2:$H$116,$A14,'Picks'!$U$2:$U$116,"settled")</f>
+        <f>COUNTIFS('Picks'!$H$2:$H$119,$A14,'Picks'!$U$2:$U$119,"settled")</f>
         <v/>
       </c>
       <c r="C14" s="13">
-        <f>COUNTIFS('Picks'!$H$2:$H$116,$A14,'Picks'!$U$2:$U$116,"settled",'Picks'!$V$2:$V$116,"win")</f>
+        <f>COUNTIFS('Picks'!$H$2:$H$119,$A14,'Picks'!$U$2:$U$119,"settled",'Picks'!$V$2:$V$119,"win")</f>
         <v/>
       </c>
       <c r="D14" s="13">
-        <f>COUNTIFS('Picks'!$H$2:$H$116,$A14,'Picks'!$U$2:$U$116,"settled",'Picks'!$V$2:$V$116,"loss")</f>
+        <f>COUNTIFS('Picks'!$H$2:$H$119,$A14,'Picks'!$U$2:$U$119,"settled",'Picks'!$V$2:$V$119,"loss")</f>
         <v/>
       </c>
       <c r="E14" s="14">
@@ -943,11 +943,11 @@
         <v/>
       </c>
       <c r="F14" s="15">
-        <f>SUMIFS('Picks'!$BY$2:$BY$116,'Picks'!$H$2:$H$116,$A14)</f>
+        <f>SUMIFS('Picks'!$BY$2:$BY$119,'Picks'!$H$2:$H$119,$A14)</f>
         <v/>
       </c>
       <c r="G14" s="16">
-        <f>IFERROR(AVERAGEIFS('Picks'!$AB$2:$AB$116,'Picks'!$H$2:$H$116,$A14,'Picks'!$U$2:$U$116,"settled"),0)</f>
+        <f>IFERROR(AVERAGEIFS('Picks'!$AB$2:$AB$119,'Picks'!$H$2:$H$119,$A14,'Picks'!$U$2:$U$119,"settled"),0)</f>
         <v/>
       </c>
     </row>
@@ -958,15 +958,15 @@
         </is>
       </c>
       <c r="B15" s="18">
-        <f>COUNTIFS('Picks'!$H$2:$H$116,$A15,'Picks'!$U$2:$U$116,"settled")</f>
+        <f>COUNTIFS('Picks'!$H$2:$H$119,$A15,'Picks'!$U$2:$U$119,"settled")</f>
         <v/>
       </c>
       <c r="C15" s="18">
-        <f>COUNTIFS('Picks'!$H$2:$H$116,$A15,'Picks'!$U$2:$U$116,"settled",'Picks'!$V$2:$V$116,"win")</f>
+        <f>COUNTIFS('Picks'!$H$2:$H$119,$A15,'Picks'!$U$2:$U$119,"settled",'Picks'!$V$2:$V$119,"win")</f>
         <v/>
       </c>
       <c r="D15" s="18">
-        <f>COUNTIFS('Picks'!$H$2:$H$116,$A15,'Picks'!$U$2:$U$116,"settled",'Picks'!$V$2:$V$116,"loss")</f>
+        <f>COUNTIFS('Picks'!$H$2:$H$119,$A15,'Picks'!$U$2:$U$119,"settled",'Picks'!$V$2:$V$119,"loss")</f>
         <v/>
       </c>
       <c r="E15" s="19">
@@ -974,11 +974,11 @@
         <v/>
       </c>
       <c r="F15" s="20">
-        <f>SUMIFS('Picks'!$BY$2:$BY$116,'Picks'!$H$2:$H$116,$A15)</f>
+        <f>SUMIFS('Picks'!$BY$2:$BY$119,'Picks'!$H$2:$H$119,$A15)</f>
         <v/>
       </c>
       <c r="G15" s="21">
-        <f>IFERROR(AVERAGEIFS('Picks'!$AB$2:$AB$116,'Picks'!$H$2:$H$116,$A15,'Picks'!$U$2:$U$116,"settled"),0)</f>
+        <f>IFERROR(AVERAGEIFS('Picks'!$AB$2:$AB$119,'Picks'!$H$2:$H$119,$A15,'Picks'!$U$2:$U$119,"settled"),0)</f>
         <v/>
       </c>
     </row>
@@ -989,15 +989,15 @@
         </is>
       </c>
       <c r="B16" s="13">
-        <f>COUNTIFS('Picks'!$H$2:$H$116,$A16,'Picks'!$U$2:$U$116,"settled")</f>
+        <f>COUNTIFS('Picks'!$H$2:$H$119,$A16,'Picks'!$U$2:$U$119,"settled")</f>
         <v/>
       </c>
       <c r="C16" s="13">
-        <f>COUNTIFS('Picks'!$H$2:$H$116,$A16,'Picks'!$U$2:$U$116,"settled",'Picks'!$V$2:$V$116,"win")</f>
+        <f>COUNTIFS('Picks'!$H$2:$H$119,$A16,'Picks'!$U$2:$U$119,"settled",'Picks'!$V$2:$V$119,"win")</f>
         <v/>
       </c>
       <c r="D16" s="13">
-        <f>COUNTIFS('Picks'!$H$2:$H$116,$A16,'Picks'!$U$2:$U$116,"settled",'Picks'!$V$2:$V$116,"loss")</f>
+        <f>COUNTIFS('Picks'!$H$2:$H$119,$A16,'Picks'!$U$2:$U$119,"settled",'Picks'!$V$2:$V$119,"loss")</f>
         <v/>
       </c>
       <c r="E16" s="14">
@@ -1005,11 +1005,11 @@
         <v/>
       </c>
       <c r="F16" s="15">
-        <f>SUMIFS('Picks'!$BY$2:$BY$116,'Picks'!$H$2:$H$116,$A16)</f>
+        <f>SUMIFS('Picks'!$BY$2:$BY$119,'Picks'!$H$2:$H$119,$A16)</f>
         <v/>
       </c>
       <c r="G16" s="16">
-        <f>IFERROR(AVERAGEIFS('Picks'!$AB$2:$AB$116,'Picks'!$H$2:$H$116,$A16,'Picks'!$U$2:$U$116,"settled"),0)</f>
+        <f>IFERROR(AVERAGEIFS('Picks'!$AB$2:$AB$119,'Picks'!$H$2:$H$119,$A16,'Picks'!$U$2:$U$119,"settled"),0)</f>
         <v/>
       </c>
     </row>
@@ -1038,7 +1038,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:DQ116"/>
+  <dimension ref="A1:DQ119"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -37608,18 +37608,38 @@
       </c>
       <c r="U114" s="24" t="inlineStr">
         <is>
-          <t>open</t>
-        </is>
-      </c>
-      <c r="V114" s="24" t="n"/>
-      <c r="W114" s="26" t="n"/>
-      <c r="X114" s="26" t="n"/>
+          <t>settled</t>
+        </is>
+      </c>
+      <c r="V114" s="24" t="inlineStr">
+        <is>
+          <t>win</t>
+        </is>
+      </c>
+      <c r="W114" s="26" t="n">
+        <v>1</v>
+      </c>
+      <c r="X114" s="26" t="n">
+        <v>0</v>
+      </c>
       <c r="Y114" s="25" t="n"/>
-      <c r="Z114" s="26" t="n"/>
-      <c r="AA114" s="28" t="n"/>
-      <c r="AB114" s="28" t="n"/>
-      <c r="AC114" s="30" t="n"/>
-      <c r="AD114" s="24" t="n"/>
+      <c r="Z114" s="26" t="n">
+        <v>-133</v>
+      </c>
+      <c r="AA114" s="28" t="n">
+        <v>0.57</v>
+      </c>
+      <c r="AB114" s="28" t="n">
+        <v>-0.000815</v>
+      </c>
+      <c r="AC114" s="30" t="n">
+        <v>0.7519</v>
+      </c>
+      <c r="AD114" s="24" t="inlineStr">
+        <is>
+          <t>2026-10-06T10:03:05.704498Z</t>
+        </is>
+      </c>
       <c r="AE114" s="31" t="inlineStr">
         <is>
           <t>Neutral Elo baseline; executable ask 0.5700 (market_slug=aec-dota2-yg-iac-2026-10-06).</t>
@@ -37762,8 +37782,12 @@
       <c r="BN114" s="28" t="n"/>
       <c r="BO114" s="28" t="n"/>
       <c r="BP114" s="25" t="n"/>
-      <c r="BQ114" s="27" t="n"/>
-      <c r="BR114" s="28" t="n"/>
+      <c r="BQ114" s="27" t="n">
+        <v>1.75188</v>
+      </c>
+      <c r="BR114" s="28" t="n">
+        <v>0.57</v>
+      </c>
       <c r="BS114" s="28" t="n"/>
       <c r="BT114" s="28" t="n"/>
       <c r="BU114" s="25" t="n"/>
@@ -37905,18 +37929,38 @@
       </c>
       <c r="U115" s="24" t="inlineStr">
         <is>
-          <t>open</t>
-        </is>
-      </c>
-      <c r="V115" s="24" t="n"/>
-      <c r="W115" s="26" t="n"/>
-      <c r="X115" s="26" t="n"/>
+          <t>settled</t>
+        </is>
+      </c>
+      <c r="V115" s="24" t="inlineStr">
+        <is>
+          <t>loss</t>
+        </is>
+      </c>
+      <c r="W115" s="26" t="n">
+        <v>1</v>
+      </c>
+      <c r="X115" s="26" t="n">
+        <v>0</v>
+      </c>
       <c r="Y115" s="25" t="n"/>
-      <c r="Z115" s="26" t="n"/>
-      <c r="AA115" s="28" t="n"/>
-      <c r="AB115" s="28" t="n"/>
-      <c r="AC115" s="30" t="n"/>
-      <c r="AD115" s="24" t="n"/>
+      <c r="Z115" s="26" t="n">
+        <v>-900</v>
+      </c>
+      <c r="AA115" s="28" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="AB115" s="28" t="n">
+        <v>0.309836</v>
+      </c>
+      <c r="AC115" s="30" t="n">
+        <v>-1</v>
+      </c>
+      <c r="AD115" s="24" t="inlineStr">
+        <is>
+          <t>2026-10-06T16:05:14.355704Z</t>
+        </is>
+      </c>
       <c r="AE115" s="31" t="inlineStr">
         <is>
           <t>Neutral Elo baseline; executable ask 0.5900 (market_slug=aec-dota2-hul-ch-2026-10-06).</t>
@@ -37929,7 +37973,7 @@
       </c>
       <c r="AG115" s="24" t="inlineStr">
         <is>
-          <t>not_applicable</t>
+          <t>review_required</t>
         </is>
       </c>
       <c r="AH115" s="24" t="n"/>
@@ -38059,8 +38103,12 @@
       <c r="BN115" s="28" t="n"/>
       <c r="BO115" s="28" t="n"/>
       <c r="BP115" s="25" t="n"/>
-      <c r="BQ115" s="27" t="n"/>
-      <c r="BR115" s="28" t="n"/>
+      <c r="BQ115" s="27" t="n">
+        <v>1.111111</v>
+      </c>
+      <c r="BR115" s="28" t="n">
+        <v>0.9</v>
+      </c>
       <c r="BS115" s="28" t="n"/>
       <c r="BT115" s="28" t="n"/>
       <c r="BU115" s="25" t="n"/>
@@ -38124,12 +38172,12 @@
     <row r="116" ht="36" customHeight="1">
       <c r="A116" s="24" t="inlineStr">
         <is>
-          <t>01e1af3dedca4d71</t>
+          <t>fd1c05e7e1ce4b8f</t>
         </is>
       </c>
       <c r="B116" s="24" t="inlineStr">
         <is>
-          <t>2026-10-05T22:25:55.486296Z</t>
+          <t>2026-10-06T10:51:23.725681Z</t>
         </is>
       </c>
       <c r="C116" s="24" t="inlineStr">
@@ -38183,11 +38231,11 @@
         <v>0.45045</v>
       </c>
       <c r="O116" s="28" t="n">
-        <v>0.587048</v>
+        <v>0.586581</v>
       </c>
       <c r="P116" s="28" t="n"/>
       <c r="Q116" s="28" t="n">
-        <v>0.136598</v>
+        <v>0.136131</v>
       </c>
       <c r="R116" s="26" t="n">
         <v>88</v>
@@ -38202,18 +38250,38 @@
       </c>
       <c r="U116" s="24" t="inlineStr">
         <is>
-          <t>open</t>
-        </is>
-      </c>
-      <c r="V116" s="24" t="n"/>
-      <c r="W116" s="26" t="n"/>
-      <c r="X116" s="26" t="n"/>
+          <t>settled</t>
+        </is>
+      </c>
+      <c r="V116" s="24" t="inlineStr">
+        <is>
+          <t>win</t>
+        </is>
+      </c>
+      <c r="W116" s="26" t="n">
+        <v>0</v>
+      </c>
+      <c r="X116" s="26" t="n">
+        <v>1</v>
+      </c>
       <c r="Y116" s="25" t="n"/>
-      <c r="Z116" s="26" t="n"/>
-      <c r="AA116" s="28" t="n"/>
-      <c r="AB116" s="28" t="n"/>
-      <c r="AC116" s="30" t="n"/>
-      <c r="AD116" s="24" t="n"/>
+      <c r="Z116" s="26" t="n">
+        <v>122</v>
+      </c>
+      <c r="AA116" s="28" t="n">
+        <v>0.45</v>
+      </c>
+      <c r="AB116" s="28" t="n">
+        <v>-0.00045</v>
+      </c>
+      <c r="AC116" s="30" t="n">
+        <v>1.83</v>
+      </c>
+      <c r="AD116" s="24" t="inlineStr">
+        <is>
+          <t>2026-10-06T22:05:25.356164Z</t>
+        </is>
+      </c>
       <c r="AE116" s="31" t="inlineStr">
         <is>
           <t>Neutral Elo baseline; executable ask 0.4500 (market_slug=aec-dota2-tsea-yes-2026-10-06).</t>
@@ -38300,7 +38368,7 @@
       </c>
       <c r="BA116" s="24" t="inlineStr">
         <is>
-          <t>8fd316347e24d5faa7a92e7ef89a639c490973a25d2b8dbb2af706a2af5abf92</t>
+          <t>6759e71c6db4f5d9b0ec78bb2474758963eb5552e8a6657a0edf8ae49f26fe3d</t>
         </is>
       </c>
       <c r="BB116" s="24" t="inlineStr">
@@ -38315,7 +38383,7 @@
       </c>
       <c r="BD116" s="24" t="inlineStr">
         <is>
-          <t>8fd316347e24d5faa7a92e7ef89a639c490973a25d2b8dbb2af706a2af5abf92</t>
+          <t>6759e71c6db4f5d9b0ec78bb2474758963eb5552e8a6657a0edf8ae49f26fe3d</t>
         </is>
       </c>
       <c r="BE116" s="24" t="inlineStr">
@@ -38335,7 +38403,7 @@
       </c>
       <c r="BH116" s="24" t="inlineStr">
         <is>
-          <t>2026-10-05T22:25:44.939151Z</t>
+          <t>2026-10-06T10:51:03.361802Z</t>
         </is>
       </c>
       <c r="BI116" s="24" t="inlineStr">
@@ -38356,8 +38424,12 @@
       <c r="BN116" s="28" t="n"/>
       <c r="BO116" s="28" t="n"/>
       <c r="BP116" s="25" t="n"/>
-      <c r="BQ116" s="27" t="n"/>
-      <c r="BR116" s="28" t="n"/>
+      <c r="BQ116" s="27" t="n">
+        <v>2.22</v>
+      </c>
+      <c r="BR116" s="28" t="n">
+        <v>0.45</v>
+      </c>
       <c r="BS116" s="28" t="n"/>
       <c r="BT116" s="28" t="n"/>
       <c r="BU116" s="25" t="n"/>
@@ -38414,7 +38486,922 @@
       <c r="DP116" s="24" t="n"/>
       <c r="DQ116" s="24" t="inlineStr">
         <is>
-          <t>{"artifact_hash": "8fd316347e24d5faa7a92e7ef89a639c490973a25d2b8dbb2af706a2af5abf92", "away_team": "Yellow Submarine", "event_id": "143565", "event_start_utc": "2026-10-06T14:00:00Z", "features": {"away_elo": 1786.068317, "away_history_count": 285, "home_elo": 1855.48017, "home_history_count": 23}, "historical_source_observation_times_verified": false, "home_team": "Team Synapse", "inference_inputs": {"book_state": {"games_played": {"bo3:4:16486": 285, "bo3:4:25201": 23}, "inactivity_half_life_days": null, "inactivity_max_pull": null, "k": 48.0, "last_match_utc": {"bo3:4:16486": "2026-10-05T11:10:00Z", "bo3:4:25201": "2026-10-05T08:00:00Z"}, "minimum_reliable_games": null, "platt_intercept": 0.08103315066152637, "platt_slope": 0.8449481325411426, "ratings": {"bo3:4:16486": 1786.068317, "bo3:4:25201": 1855.48017}, "recency_half_life_days": null, "recency_max_boost": null, "temperature": 1.18, "thin_data_max_shrink": null, "tier_weights": null}, "code_sha256": {"esports.py": "48eab29fd660f72bcbd6f9557cca081a5e6f76c9da89c9cf36ce7181c79b1174", "features/elo_ratings.py": "8525faf022a6343c452286dbfeb17dbb043744c6bdabbe448b6b371216da439b"}, "reference_date": "2026-10-05T22:25:23.694580+00:00", "team_ids": ["bo3:4:25201", "bo3:4:16486"]}, "market_type": "moneyline", "model_version": "dota2-tiered-elo-v6", "observed_at_utc": "2026-10-05T22:25:23.694580+00:00", "probabilities": {"away": 0.412952, "home": 0.587048}, "replay_scope": "Exact serving book state, calibration, temperature, inactivity reference and thin-history adjustments; training provenance not certified.", "schema": "esports-elo-replay-v1", "snapshot_hash": "de1d70f15f33b8dcda068e21a4a94c374808390850c2e0df4df0409544cc1b27", "sport": "DOTA2"}</t>
+          <t>{"artifact_hash": "6759e71c6db4f5d9b0ec78bb2474758963eb5552e8a6657a0edf8ae49f26fe3d", "away_team": "Yellow Submarine", "event_id": "143565", "event_start_utc": "2026-10-06T14:00:00Z", "features": {"away_elo": 1786.028424, "away_history_count": 285, "home_elo": 1855.458017, "home_history_count": 23}, "historical_source_observation_times_verified": false, "home_team": "Team Synapse", "inference_inputs": {"book_state": {"games_played": {"bo3:4:16486": 285, "bo3:4:25201": 23}, "inactivity_half_life_days": null, "inactivity_max_pull": null, "k": 48.0, "last_match_utc": {"bo3:4:16486": "2026-10-05T11:10:00Z", "bo3:4:25201": "2026-10-05T08:00:00Z"}, "minimum_reliable_games": null, "platt_intercept": 0.0806649303548175, "platt_slope": 0.8439015098774778, "ratings": {"bo3:4:16486": 1786.028424, "bo3:4:25201": 1855.458017}, "recency_half_life_days": null, "recency_max_boost": null, "temperature": 1.18, "thin_data_max_shrink": null, "tier_weights": null}, "code_sha256": {"esports.py": "48eab29fd660f72bcbd6f9557cca081a5e6f76c9da89c9cf36ce7181c79b1174", "features/elo_ratings.py": "8525faf022a6343c452286dbfeb17dbb043744c6bdabbe448b6b371216da439b"}, "reference_date": "2026-10-06T10:50:53.111088+00:00", "team_ids": ["bo3:4:25201", "bo3:4:16486"]}, "market_type": "moneyline", "model_version": "dota2-tiered-elo-v6", "observed_at_utc": "2026-10-06T10:50:53.111088+00:00", "probabilities": {"away": 0.413419, "home": 0.586581}, "replay_scope": "Exact serving book state, calibration, temperature, inactivity reference and thin-history adjustments; training provenance not certified.", "schema": "esports-elo-replay-v1", "snapshot_hash": "2d95927cb9101c0d665d6d64969b5ac62cd066f6a48af941c35e0f56d54aa876", "sport": "DOTA2"}</t>
+        </is>
+      </c>
+    </row>
+    <row r="117" ht="36" customHeight="1">
+      <c r="A117" s="24" t="inlineStr">
+        <is>
+          <t>120dd1ec1cd24c81</t>
+        </is>
+      </c>
+      <c r="B117" s="24" t="inlineStr">
+        <is>
+          <t>2026-10-06T16:34:32.687894Z</t>
+        </is>
+      </c>
+      <c r="C117" s="24" t="inlineStr">
+        <is>
+          <t>2026-10-06T17:00:00Z</t>
+        </is>
+      </c>
+      <c r="D117" s="24" t="inlineStr">
+        <is>
+          <t>144500</t>
+        </is>
+      </c>
+      <c r="E117" s="24" t="inlineStr">
+        <is>
+          <t>DOTA2</t>
+        </is>
+      </c>
+      <c r="F117" s="24" t="inlineStr">
+        <is>
+          <t>MOUZ</t>
+        </is>
+      </c>
+      <c r="G117" s="24" t="inlineStr">
+        <is>
+          <t>LEGION</t>
+        </is>
+      </c>
+      <c r="H117" s="24" t="inlineStr">
+        <is>
+          <t>moneyline</t>
+        </is>
+      </c>
+      <c r="I117" s="24" t="inlineStr">
+        <is>
+          <t>away</t>
+        </is>
+      </c>
+      <c r="J117" s="25" t="n"/>
+      <c r="K117" s="24" t="inlineStr">
+        <is>
+          <t>polymarket_us</t>
+        </is>
+      </c>
+      <c r="L117" s="26" t="n">
+        <v>-117</v>
+      </c>
+      <c r="M117" s="27" t="n">
+        <v>1.854701</v>
+      </c>
+      <c r="N117" s="28" t="n">
+        <v>0.539171</v>
+      </c>
+      <c r="O117" s="28" t="n">
+        <v>0.552316</v>
+      </c>
+      <c r="P117" s="28" t="n"/>
+      <c r="Q117" s="28" t="n">
+        <v>0.013145</v>
+      </c>
+      <c r="R117" s="26" t="n">
+        <v>27</v>
+      </c>
+      <c r="S117" s="29" t="n">
+        <v>1</v>
+      </c>
+      <c r="T117" s="24" t="inlineStr">
+        <is>
+          <t>dota2-tiered-elo-v6</t>
+        </is>
+      </c>
+      <c r="U117" s="24" t="inlineStr">
+        <is>
+          <t>settled</t>
+        </is>
+      </c>
+      <c r="V117" s="24" t="inlineStr">
+        <is>
+          <t>loss</t>
+        </is>
+      </c>
+      <c r="W117" s="26" t="n">
+        <v>0</v>
+      </c>
+      <c r="X117" s="26" t="n">
+        <v>1</v>
+      </c>
+      <c r="Y117" s="25" t="n"/>
+      <c r="Z117" s="26" t="n">
+        <v>-117</v>
+      </c>
+      <c r="AA117" s="28" t="n">
+        <v>0.54</v>
+      </c>
+      <c r="AB117" s="28" t="n">
+        <v>0.000829</v>
+      </c>
+      <c r="AC117" s="30" t="n">
+        <v>-1</v>
+      </c>
+      <c r="AD117" s="24" t="inlineStr">
+        <is>
+          <t>2026-10-06T22:05:27.593158Z</t>
+        </is>
+      </c>
+      <c r="AE117" s="31" t="inlineStr">
+        <is>
+          <t>Neutral Elo baseline; executable ask 0.5400 (market_slug=aec-dota2-leg-mouz-2026-10-06).</t>
+        </is>
+      </c>
+      <c r="AF117" s="31" t="inlineStr">
+        <is>
+          <t>Config-promoted esports baseline; gates enforced at log time.</t>
+        </is>
+      </c>
+      <c r="AG117" s="24" t="inlineStr">
+        <is>
+          <t>review_required</t>
+        </is>
+      </c>
+      <c r="AH117" s="24" t="n"/>
+      <c r="AI117" s="31" t="n"/>
+      <c r="AJ117" s="31" t="n"/>
+      <c r="AK117" s="24" t="inlineStr">
+        <is>
+          <t>paper_call</t>
+        </is>
+      </c>
+      <c r="AL117" s="26" t="n">
+        <v>4</v>
+      </c>
+      <c r="AM117" s="24" t="inlineStr">
+        <is>
+          <t>RESEARCH_OBSERVATION</t>
+        </is>
+      </c>
+      <c r="AN117" s="24" t="inlineStr">
+        <is>
+          <t>CALL</t>
+        </is>
+      </c>
+      <c r="AO117" s="24" t="inlineStr">
+        <is>
+          <t>PAPER_CALL_LOW_EDGE</t>
+        </is>
+      </c>
+      <c r="AP117" s="24" t="inlineStr">
+        <is>
+          <t>MOUZ</t>
+        </is>
+      </c>
+      <c r="AQ117" s="24" t="inlineStr">
+        <is>
+          <t>MOUZ</t>
+        </is>
+      </c>
+      <c r="AR117" s="24" t="inlineStr">
+        <is>
+          <t>MOUZ</t>
+        </is>
+      </c>
+      <c r="AS117" s="24" t="inlineStr">
+        <is>
+          <t>LEGION</t>
+        </is>
+      </c>
+      <c r="AT117" s="24" t="inlineStr">
+        <is>
+          <t>LEGION</t>
+        </is>
+      </c>
+      <c r="AU117" s="24" t="inlineStr">
+        <is>
+          <t>LEGION</t>
+        </is>
+      </c>
+      <c r="AV117" s="24" t="n"/>
+      <c r="AW117" s="24" t="n"/>
+      <c r="AX117" s="24" t="inlineStr">
+        <is>
+          <t>statistical_model</t>
+        </is>
+      </c>
+      <c r="AY117" s="24" t="n"/>
+      <c r="AZ117" s="24" t="inlineStr">
+        <is>
+          <t>shadow_qualified</t>
+        </is>
+      </c>
+      <c r="BA117" s="24" t="inlineStr">
+        <is>
+          <t>4690b99c58f0ec38c0a7f8871260c2693630b47ca56007141cc547de632674ee</t>
+        </is>
+      </c>
+      <c r="BB117" s="24" t="inlineStr">
+        <is>
+          <t>neutral_elo</t>
+        </is>
+      </c>
+      <c r="BC117" s="24" t="inlineStr">
+        <is>
+          <t>dota2-tiered-elo-v6</t>
+        </is>
+      </c>
+      <c r="BD117" s="24" t="inlineStr">
+        <is>
+          <t>4690b99c58f0ec38c0a7f8871260c2693630b47ca56007141cc547de632674ee</t>
+        </is>
+      </c>
+      <c r="BE117" s="24" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="BF117" s="24" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="BG117" s="24" t="inlineStr">
+        <is>
+          <t>dota2-tiered-elo-v6</t>
+        </is>
+      </c>
+      <c r="BH117" s="24" t="inlineStr">
+        <is>
+          <t>2026-10-06T16:34:12.398493Z</t>
+        </is>
+      </c>
+      <c r="BI117" s="24" t="inlineStr">
+        <is>
+          <t>["same_event","same_team_same_day","same_league_same_day"]</t>
+        </is>
+      </c>
+      <c r="BJ117" s="25" t="n"/>
+      <c r="BK117" s="26" t="n">
+        <v>-117</v>
+      </c>
+      <c r="BL117" s="27" t="n">
+        <v>1.854701</v>
+      </c>
+      <c r="BM117" s="28" t="n">
+        <v>0.539171</v>
+      </c>
+      <c r="BN117" s="28" t="n"/>
+      <c r="BO117" s="28" t="n"/>
+      <c r="BP117" s="25" t="n"/>
+      <c r="BQ117" s="27" t="n">
+        <v>1.854701</v>
+      </c>
+      <c r="BR117" s="28" t="n">
+        <v>0.54</v>
+      </c>
+      <c r="BS117" s="28" t="n"/>
+      <c r="BT117" s="28" t="n"/>
+      <c r="BU117" s="25" t="n"/>
+      <c r="BV117" s="29" t="n"/>
+      <c r="BW117" s="24" t="n"/>
+      <c r="BX117" s="30" t="n"/>
+      <c r="BY117" s="27" t="n"/>
+      <c r="BZ117" s="24" t="n"/>
+      <c r="CA117" s="31" t="n"/>
+      <c r="CB117" s="24" t="n"/>
+      <c r="CC117" s="24" t="n"/>
+      <c r="CD117" s="24" t="n"/>
+      <c r="CE117" s="24" t="n"/>
+      <c r="CF117" s="24" t="n"/>
+      <c r="CG117" s="24" t="n"/>
+      <c r="CH117" s="24" t="n"/>
+      <c r="CI117" s="24" t="n"/>
+      <c r="CJ117" s="24" t="n"/>
+      <c r="CK117" s="24" t="n"/>
+      <c r="CL117" s="24" t="n"/>
+      <c r="CM117" s="24" t="n"/>
+      <c r="CN117" s="24" t="n"/>
+      <c r="CO117" s="24" t="n"/>
+      <c r="CP117" s="24" t="n"/>
+      <c r="CQ117" s="24" t="n"/>
+      <c r="CR117" s="24" t="n"/>
+      <c r="CS117" s="24" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="CT117" s="24" t="n"/>
+      <c r="CU117" s="24" t="n"/>
+      <c r="CV117" s="24" t="n"/>
+      <c r="CW117" s="24" t="n"/>
+      <c r="CX117" s="24" t="n"/>
+      <c r="CY117" s="24" t="n"/>
+      <c r="CZ117" s="24" t="n"/>
+      <c r="DA117" s="24" t="n"/>
+      <c r="DB117" s="24" t="n"/>
+      <c r="DC117" s="24" t="n"/>
+      <c r="DD117" s="24" t="n"/>
+      <c r="DE117" s="24" t="n"/>
+      <c r="DF117" s="24" t="n"/>
+      <c r="DG117" s="24" t="n"/>
+      <c r="DH117" s="24" t="n"/>
+      <c r="DI117" s="24" t="n"/>
+      <c r="DJ117" s="24" t="n"/>
+      <c r="DK117" s="24" t="n"/>
+      <c r="DL117" s="24" t="n"/>
+      <c r="DM117" s="24" t="n"/>
+      <c r="DN117" s="24" t="n"/>
+      <c r="DO117" s="24" t="n"/>
+      <c r="DP117" s="24" t="n"/>
+      <c r="DQ117" s="24" t="inlineStr">
+        <is>
+          <t>{"artifact_hash": "4690b99c58f0ec38c0a7f8871260c2693630b47ca56007141cc547de632674ee", "away_team": "MOUZ", "event_id": "144500", "event_start_utc": "2026-10-06T17:00:00Z", "features": {"away_elo": 1644.197963, "away_history_count": 363, "home_elo": 1532.76, "home_history_count": 1}, "historical_source_observation_times_verified": false, "home_team": "LEGION", "inference_inputs": {"book_state": {"games_played": {"bo3:4:15032": 363, "bo3:4:25401": 1}, "inactivity_half_life_days": null, "inactivity_max_pull": null, "k": 48.0, "last_match_utc": {"bo3:4:15032": "2026-10-05T18:00:00Z", "bo3:4:25401": "2026-10-05T14:00:00Z"}, "minimum_reliable_games": null, "platt_intercept": 0.08111949537955908, "platt_slope": 0.8418535477548365, "ratings": {"bo3:4:15032": 1644.197963, "bo3:4:25401": 1532.76}, "recency_half_life_days": null, "recency_max_boost": null, "temperature": 1.18, "thin_data_max_shrink": null, "tier_weights": null}, "code_sha256": {"esports.py": "48eab29fd660f72bcbd6f9557cca081a5e6f76c9da89c9cf36ce7181c79b1174", "features/elo_ratings.py": "8525faf022a6343c452286dbfeb17dbb043744c6bdabbe448b6b371216da439b"}, "reference_date": "2026-10-06T16:34:12.325280+00:00", "team_ids": ["bo3:4:25401", "bo3:4:15032"]}, "market_type": "moneyline", "model_version": "dota2-tiered-elo-v6", "observed_at_utc": "2026-10-06T16:34:12.325280+00:00", "probabilities": {"away": 0.552316, "home": 0.447684}, "replay_scope": "Exact serving book state, calibration, temperature, inactivity reference and thin-history adjustments; training provenance not certified.", "schema": "esports-elo-replay-v1", "snapshot_hash": "d7ab51a4f880e3c1e54ff9e61bc180831b900208cf5f6dcb73682f2580b1dd3d", "sport": "DOTA2"}</t>
+        </is>
+      </c>
+    </row>
+    <row r="118" ht="36" customHeight="1">
+      <c r="A118" s="24" t="inlineStr">
+        <is>
+          <t>e78ebb127f8b4a80</t>
+        </is>
+      </c>
+      <c r="B118" s="24" t="inlineStr">
+        <is>
+          <t>2026-10-06T22:25:56.390271Z</t>
+        </is>
+      </c>
+      <c r="C118" s="24" t="inlineStr">
+        <is>
+          <t>2026-10-07T03:00:00Z</t>
+        </is>
+      </c>
+      <c r="D118" s="24" t="inlineStr">
+        <is>
+          <t>145226</t>
+        </is>
+      </c>
+      <c r="E118" s="24" t="inlineStr">
+        <is>
+          <t>DOTA2</t>
+        </is>
+      </c>
+      <c r="F118" s="24" t="inlineStr">
+        <is>
+          <t>ЯЧЁ123</t>
+        </is>
+      </c>
+      <c r="G118" s="24" t="inlineStr">
+        <is>
+          <t>Direborn</t>
+        </is>
+      </c>
+      <c r="H118" s="24" t="inlineStr">
+        <is>
+          <t>moneyline</t>
+        </is>
+      </c>
+      <c r="I118" s="24" t="inlineStr">
+        <is>
+          <t>home</t>
+        </is>
+      </c>
+      <c r="J118" s="25" t="n"/>
+      <c r="K118" s="24" t="inlineStr">
+        <is>
+          <t>polymarket_us</t>
+        </is>
+      </c>
+      <c r="L118" s="26" t="n">
+        <v>-233</v>
+      </c>
+      <c r="M118" s="27" t="n">
+        <v>1.429185</v>
+      </c>
+      <c r="N118" s="28" t="n">
+        <v>0.6997</v>
+      </c>
+      <c r="O118" s="28" t="n">
+        <v>0.550796</v>
+      </c>
+      <c r="P118" s="28" t="n"/>
+      <c r="Q118" s="28" t="n">
+        <v>-0.148904</v>
+      </c>
+      <c r="R118" s="26" t="n">
+        <v>0</v>
+      </c>
+      <c r="S118" s="29" t="n">
+        <v>1</v>
+      </c>
+      <c r="T118" s="24" t="inlineStr">
+        <is>
+          <t>dota2-tiered-elo-v6</t>
+        </is>
+      </c>
+      <c r="U118" s="24" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="V118" s="24" t="n"/>
+      <c r="W118" s="26" t="n"/>
+      <c r="X118" s="26" t="n"/>
+      <c r="Y118" s="25" t="n"/>
+      <c r="Z118" s="26" t="n"/>
+      <c r="AA118" s="28" t="n"/>
+      <c r="AB118" s="28" t="n"/>
+      <c r="AC118" s="30" t="n"/>
+      <c r="AD118" s="24" t="n"/>
+      <c r="AE118" s="31" t="inlineStr">
+        <is>
+          <t>Neutral Elo baseline; executable ask 0.7000 (market_slug=aec-dota2-db-y123-2026-10-07).</t>
+        </is>
+      </c>
+      <c r="AF118" s="31" t="inlineStr">
+        <is>
+          <t>Config-promoted esports baseline; gates enforced at log time.</t>
+        </is>
+      </c>
+      <c r="AG118" s="24" t="inlineStr">
+        <is>
+          <t>not_applicable</t>
+        </is>
+      </c>
+      <c r="AH118" s="24" t="n"/>
+      <c r="AI118" s="31" t="n"/>
+      <c r="AJ118" s="31" t="n"/>
+      <c r="AK118" s="24" t="inlineStr">
+        <is>
+          <t>paper_call</t>
+        </is>
+      </c>
+      <c r="AL118" s="26" t="n">
+        <v>4</v>
+      </c>
+      <c r="AM118" s="24" t="inlineStr">
+        <is>
+          <t>RESEARCH_OBSERVATION</t>
+        </is>
+      </c>
+      <c r="AN118" s="24" t="inlineStr">
+        <is>
+          <t>CALL</t>
+        </is>
+      </c>
+      <c r="AO118" s="24" t="inlineStr">
+        <is>
+          <t>PAPER_CALL_MODEL_UNVALIDATED</t>
+        </is>
+      </c>
+      <c r="AP118" s="24" t="inlineStr">
+        <is>
+          <t>ЯЧЁ123</t>
+        </is>
+      </c>
+      <c r="AQ118" s="24" t="inlineStr">
+        <is>
+          <t>ЯЧЁ123</t>
+        </is>
+      </c>
+      <c r="AR118" s="24" t="inlineStr">
+        <is>
+          <t>ЯЧЁ123</t>
+        </is>
+      </c>
+      <c r="AS118" s="24" t="inlineStr">
+        <is>
+          <t>Direborn</t>
+        </is>
+      </c>
+      <c r="AT118" s="24" t="inlineStr">
+        <is>
+          <t>Direborn</t>
+        </is>
+      </c>
+      <c r="AU118" s="24" t="inlineStr">
+        <is>
+          <t>Direborn</t>
+        </is>
+      </c>
+      <c r="AV118" s="24" t="n"/>
+      <c r="AW118" s="24" t="n"/>
+      <c r="AX118" s="24" t="inlineStr">
+        <is>
+          <t>statistical_model</t>
+        </is>
+      </c>
+      <c r="AY118" s="24" t="n"/>
+      <c r="AZ118" s="24" t="inlineStr">
+        <is>
+          <t>shadow_qualified</t>
+        </is>
+      </c>
+      <c r="BA118" s="24" t="inlineStr">
+        <is>
+          <t>c6996bf486b3088429204679c4a6b5d24c63cbcf4cadb3e51613f46a7fcb8642</t>
+        </is>
+      </c>
+      <c r="BB118" s="24" t="inlineStr">
+        <is>
+          <t>neutral_elo</t>
+        </is>
+      </c>
+      <c r="BC118" s="24" t="inlineStr">
+        <is>
+          <t>dota2-tiered-elo-v6</t>
+        </is>
+      </c>
+      <c r="BD118" s="24" t="inlineStr">
+        <is>
+          <t>c6996bf486b3088429204679c4a6b5d24c63cbcf4cadb3e51613f46a7fcb8642</t>
+        </is>
+      </c>
+      <c r="BE118" s="24" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="BF118" s="24" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="BG118" s="24" t="inlineStr">
+        <is>
+          <t>dota2-tiered-elo-v6</t>
+        </is>
+      </c>
+      <c r="BH118" s="24" t="inlineStr">
+        <is>
+          <t>2026-10-06T22:25:25.556351Z</t>
+        </is>
+      </c>
+      <c r="BI118" s="24" t="inlineStr">
+        <is>
+          <t>["same_event","same_team_same_day","same_league_same_day"]</t>
+        </is>
+      </c>
+      <c r="BJ118" s="25" t="n"/>
+      <c r="BK118" s="26" t="n">
+        <v>-233</v>
+      </c>
+      <c r="BL118" s="27" t="n">
+        <v>1.429185</v>
+      </c>
+      <c r="BM118" s="28" t="n">
+        <v>0.6997</v>
+      </c>
+      <c r="BN118" s="28" t="n"/>
+      <c r="BO118" s="28" t="n"/>
+      <c r="BP118" s="25" t="n"/>
+      <c r="BQ118" s="27" t="n"/>
+      <c r="BR118" s="28" t="n"/>
+      <c r="BS118" s="28" t="n"/>
+      <c r="BT118" s="28" t="n"/>
+      <c r="BU118" s="25" t="n"/>
+      <c r="BV118" s="29" t="n"/>
+      <c r="BW118" s="24" t="n"/>
+      <c r="BX118" s="30" t="n"/>
+      <c r="BY118" s="27" t="n"/>
+      <c r="BZ118" s="24" t="n"/>
+      <c r="CA118" s="31" t="n"/>
+      <c r="CB118" s="24" t="n"/>
+      <c r="CC118" s="24" t="n"/>
+      <c r="CD118" s="24" t="n"/>
+      <c r="CE118" s="24" t="n"/>
+      <c r="CF118" s="24" t="n"/>
+      <c r="CG118" s="24" t="n"/>
+      <c r="CH118" s="24" t="n"/>
+      <c r="CI118" s="24" t="n"/>
+      <c r="CJ118" s="24" t="n"/>
+      <c r="CK118" s="24" t="n"/>
+      <c r="CL118" s="24" t="n"/>
+      <c r="CM118" s="24" t="n"/>
+      <c r="CN118" s="24" t="n"/>
+      <c r="CO118" s="24" t="n"/>
+      <c r="CP118" s="24" t="n"/>
+      <c r="CQ118" s="24" t="n"/>
+      <c r="CR118" s="24" t="n"/>
+      <c r="CS118" s="24" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
+      <c r="CT118" s="24" t="n"/>
+      <c r="CU118" s="24" t="n"/>
+      <c r="CV118" s="24" t="n"/>
+      <c r="CW118" s="24" t="n"/>
+      <c r="CX118" s="24" t="n"/>
+      <c r="CY118" s="24" t="n"/>
+      <c r="CZ118" s="24" t="n"/>
+      <c r="DA118" s="24" t="n"/>
+      <c r="DB118" s="24" t="n"/>
+      <c r="DC118" s="24" t="n"/>
+      <c r="DD118" s="24" t="n"/>
+      <c r="DE118" s="24" t="n"/>
+      <c r="DF118" s="24" t="n"/>
+      <c r="DG118" s="24" t="n"/>
+      <c r="DH118" s="24" t="n"/>
+      <c r="DI118" s="24" t="n"/>
+      <c r="DJ118" s="24" t="n"/>
+      <c r="DK118" s="24" t="n"/>
+      <c r="DL118" s="24" t="n"/>
+      <c r="DM118" s="24" t="n"/>
+      <c r="DN118" s="24" t="n"/>
+      <c r="DO118" s="24" t="n"/>
+      <c r="DP118" s="24" t="n"/>
+      <c r="DQ118" s="24" t="inlineStr">
+        <is>
+          <t>{"artifact_hash": "c6996bf486b3088429204679c4a6b5d24c63cbcf4cadb3e51613f46a7fcb8642", "away_team": "\u042f\u0427\u0401123", "event_id": "145226", "event_start_utc": "2026-10-07T03:00:00Z", "features": {"away_elo": 1500.0, "away_history_count": 0, "home_elo": 1584.551416, "home_history_count": 37}, "historical_source_observation_times_verified": false, "home_team": "Direborn", "inference_inputs": {"book_state": {"games_played": {"bo3:4:24344": 37}, "inactivity_half_life_days": null, "inactivity_max_pull": null, "k": 48.0, "last_match_utc": {"bo3:4:24344": "2026-10-06T06:30:00Z"}, "minimum_reliable_games": null, "platt_intercept": 0.07646024717646603, "platt_slope": 0.8471774676108041, "ratings": {"bo3:4:24344": 1584.551416}, "recency_half_life_days": null, "recency_max_boost": null, "temperature": 1.18, "thin_data_max_shrink": null, "tier_weights": null}, "code_sha256": {"esports.py": "48eab29fd660f72bcbd6f9557cca081a5e6f76c9da89c9cf36ce7181c79b1174", "features/elo_ratings.py": "8525faf022a6343c452286dbfeb17dbb043744c6bdabbe448b6b371216da439b"}, "reference_date": "2026-10-06T22:25:25.483347+00:00", "team_ids": ["bo3:4:24344", "unknown:\u044f\u0447\u0435123"]}, "market_type": "moneyline", "model_version": "dota2-tiered-elo-v6", "observed_at_utc": "2026-10-06T22:25:25.483347+00:00", "probabilities": {"away": 0.449204, "home": 0.550796}, "replay_scope": "Exact serving book state, calibration, temperature, inactivity reference and thin-history adjustments; training provenance not certified.", "schema": "esports-elo-replay-v1", "snapshot_hash": "dc330291efd584143729f621ac5b58f7d873a090a9b0f169c927e0ebb9493b25", "sport": "DOTA2"}</t>
+        </is>
+      </c>
+    </row>
+    <row r="119" ht="36" customHeight="1">
+      <c r="A119" s="24" t="inlineStr">
+        <is>
+          <t>ae99ce3a6fdb417f</t>
+        </is>
+      </c>
+      <c r="B119" s="24" t="inlineStr">
+        <is>
+          <t>2026-10-06T22:25:56.390271Z</t>
+        </is>
+      </c>
+      <c r="C119" s="24" t="inlineStr">
+        <is>
+          <t>2026-10-07T09:00:00Z</t>
+        </is>
+      </c>
+      <c r="D119" s="24" t="inlineStr">
+        <is>
+          <t>145796</t>
+        </is>
+      </c>
+      <c r="E119" s="24" t="inlineStr">
+        <is>
+          <t>DOTA2</t>
+        </is>
+      </c>
+      <c r="F119" s="24" t="inlineStr">
+        <is>
+          <t>Yellow Submarine</t>
+        </is>
+      </c>
+      <c r="G119" s="24" t="inlineStr">
+        <is>
+          <t>Blasterbl</t>
+        </is>
+      </c>
+      <c r="H119" s="24" t="inlineStr">
+        <is>
+          <t>moneyline</t>
+        </is>
+      </c>
+      <c r="I119" s="24" t="inlineStr">
+        <is>
+          <t>away</t>
+        </is>
+      </c>
+      <c r="J119" s="25" t="n"/>
+      <c r="K119" s="24" t="inlineStr">
+        <is>
+          <t>polymarket_us</t>
+        </is>
+      </c>
+      <c r="L119" s="26" t="n">
+        <v>-156</v>
+      </c>
+      <c r="M119" s="27" t="n">
+        <v>1.641026</v>
+      </c>
+      <c r="N119" s="28" t="n">
+        <v>0.609375</v>
+      </c>
+      <c r="O119" s="28" t="n">
+        <v>0.640253</v>
+      </c>
+      <c r="P119" s="28" t="n"/>
+      <c r="Q119" s="28" t="n">
+        <v>0.030878</v>
+      </c>
+      <c r="R119" s="26" t="n">
+        <v>35</v>
+      </c>
+      <c r="S119" s="29" t="n">
+        <v>1</v>
+      </c>
+      <c r="T119" s="24" t="inlineStr">
+        <is>
+          <t>dota2-tiered-elo-v6</t>
+        </is>
+      </c>
+      <c r="U119" s="24" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="V119" s="24" t="n"/>
+      <c r="W119" s="26" t="n"/>
+      <c r="X119" s="26" t="n"/>
+      <c r="Y119" s="25" t="n"/>
+      <c r="Z119" s="26" t="n"/>
+      <c r="AA119" s="28" t="n"/>
+      <c r="AB119" s="28" t="n"/>
+      <c r="AC119" s="30" t="n"/>
+      <c r="AD119" s="24" t="n"/>
+      <c r="AE119" s="31" t="inlineStr">
+        <is>
+          <t>Neutral Elo baseline; executable ask 0.6100 (market_slug=aec-dota2-bbl-yes-2026-10-07).</t>
+        </is>
+      </c>
+      <c r="AF119" s="31" t="inlineStr">
+        <is>
+          <t>Config-promoted esports baseline; gates enforced at log time.</t>
+        </is>
+      </c>
+      <c r="AG119" s="24" t="inlineStr">
+        <is>
+          <t>not_applicable</t>
+        </is>
+      </c>
+      <c r="AH119" s="24" t="n"/>
+      <c r="AI119" s="31" t="n"/>
+      <c r="AJ119" s="31" t="n"/>
+      <c r="AK119" s="24" t="inlineStr">
+        <is>
+          <t>model_qualified</t>
+        </is>
+      </c>
+      <c r="AL119" s="26" t="n">
+        <v>4</v>
+      </c>
+      <c r="AM119" s="24" t="inlineStr">
+        <is>
+          <t>QUALIFIED_SHADOW_CALL</t>
+        </is>
+      </c>
+      <c r="AN119" s="24" t="inlineStr">
+        <is>
+          <t>CALL</t>
+        </is>
+      </c>
+      <c r="AO119" s="24" t="inlineStr">
+        <is>
+          <t>QUALIFIED</t>
+        </is>
+      </c>
+      <c r="AP119" s="24" t="inlineStr">
+        <is>
+          <t>Yellow Submarine</t>
+        </is>
+      </c>
+      <c r="AQ119" s="24" t="inlineStr">
+        <is>
+          <t>Yellow Submarine</t>
+        </is>
+      </c>
+      <c r="AR119" s="24" t="inlineStr">
+        <is>
+          <t>Yellow Submarine</t>
+        </is>
+      </c>
+      <c r="AS119" s="24" t="inlineStr">
+        <is>
+          <t>Blasterbl</t>
+        </is>
+      </c>
+      <c r="AT119" s="24" t="inlineStr">
+        <is>
+          <t>Blasterbl</t>
+        </is>
+      </c>
+      <c r="AU119" s="24" t="inlineStr">
+        <is>
+          <t>Blasterbl</t>
+        </is>
+      </c>
+      <c r="AV119" s="24" t="n"/>
+      <c r="AW119" s="24" t="n"/>
+      <c r="AX119" s="24" t="inlineStr">
+        <is>
+          <t>statistical_model</t>
+        </is>
+      </c>
+      <c r="AY119" s="24" t="n"/>
+      <c r="AZ119" s="24" t="inlineStr">
+        <is>
+          <t>shadow_qualified</t>
+        </is>
+      </c>
+      <c r="BA119" s="24" t="inlineStr">
+        <is>
+          <t>c6996bf486b3088429204679c4a6b5d24c63cbcf4cadb3e51613f46a7fcb8642</t>
+        </is>
+      </c>
+      <c r="BB119" s="24" t="inlineStr">
+        <is>
+          <t>neutral_elo</t>
+        </is>
+      </c>
+      <c r="BC119" s="24" t="inlineStr">
+        <is>
+          <t>dota2-tiered-elo-v6</t>
+        </is>
+      </c>
+      <c r="BD119" s="24" t="inlineStr">
+        <is>
+          <t>c6996bf486b3088429204679c4a6b5d24c63cbcf4cadb3e51613f46a7fcb8642</t>
+        </is>
+      </c>
+      <c r="BE119" s="24" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="BF119" s="24" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="BG119" s="24" t="inlineStr">
+        <is>
+          <t>dota2-tiered-elo-v6</t>
+        </is>
+      </c>
+      <c r="BH119" s="24" t="inlineStr">
+        <is>
+          <t>2026-10-06T22:25:25.683597Z</t>
+        </is>
+      </c>
+      <c r="BI119" s="24" t="inlineStr">
+        <is>
+          <t>["same_event","same_team_same_day","same_league_same_day"]</t>
+        </is>
+      </c>
+      <c r="BJ119" s="25" t="n"/>
+      <c r="BK119" s="26" t="n">
+        <v>-156</v>
+      </c>
+      <c r="BL119" s="27" t="n">
+        <v>1.641026</v>
+      </c>
+      <c r="BM119" s="28" t="n">
+        <v>0.609375</v>
+      </c>
+      <c r="BN119" s="28" t="n"/>
+      <c r="BO119" s="28" t="n"/>
+      <c r="BP119" s="25" t="n"/>
+      <c r="BQ119" s="27" t="n"/>
+      <c r="BR119" s="28" t="n"/>
+      <c r="BS119" s="28" t="n"/>
+      <c r="BT119" s="28" t="n"/>
+      <c r="BU119" s="25" t="n"/>
+      <c r="BV119" s="29" t="n"/>
+      <c r="BW119" s="24" t="n"/>
+      <c r="BX119" s="30" t="n"/>
+      <c r="BY119" s="27" t="n"/>
+      <c r="BZ119" s="24" t="n"/>
+      <c r="CA119" s="31" t="n"/>
+      <c r="CB119" s="24" t="n"/>
+      <c r="CC119" s="24" t="n"/>
+      <c r="CD119" s="24" t="n"/>
+      <c r="CE119" s="24" t="n"/>
+      <c r="CF119" s="24" t="n"/>
+      <c r="CG119" s="24" t="n"/>
+      <c r="CH119" s="24" t="n"/>
+      <c r="CI119" s="24" t="n"/>
+      <c r="CJ119" s="24" t="n"/>
+      <c r="CK119" s="24" t="n"/>
+      <c r="CL119" s="24" t="n"/>
+      <c r="CM119" s="24" t="n"/>
+      <c r="CN119" s="24" t="n"/>
+      <c r="CO119" s="24" t="n"/>
+      <c r="CP119" s="24" t="n"/>
+      <c r="CQ119" s="24" t="n"/>
+      <c r="CR119" s="24" t="n"/>
+      <c r="CS119" s="24" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="CT119" s="24" t="n"/>
+      <c r="CU119" s="24" t="n"/>
+      <c r="CV119" s="24" t="n"/>
+      <c r="CW119" s="24" t="n"/>
+      <c r="CX119" s="24" t="n"/>
+      <c r="CY119" s="24" t="n"/>
+      <c r="CZ119" s="24" t="n"/>
+      <c r="DA119" s="24" t="n"/>
+      <c r="DB119" s="24" t="n"/>
+      <c r="DC119" s="24" t="n"/>
+      <c r="DD119" s="24" t="n"/>
+      <c r="DE119" s="24" t="n"/>
+      <c r="DF119" s="24" t="n"/>
+      <c r="DG119" s="24" t="n"/>
+      <c r="DH119" s="24" t="n"/>
+      <c r="DI119" s="24" t="n"/>
+      <c r="DJ119" s="24" t="n"/>
+      <c r="DK119" s="24" t="n"/>
+      <c r="DL119" s="24" t="n"/>
+      <c r="DM119" s="24" t="n"/>
+      <c r="DN119" s="24" t="n"/>
+      <c r="DO119" s="24" t="n"/>
+      <c r="DP119" s="24" t="n"/>
+      <c r="DQ119" s="24" t="inlineStr">
+        <is>
+          <t>{"artifact_hash": "c6996bf486b3088429204679c4a6b5d24c63cbcf4cadb3e51613f46a7fcb8642", "away_team": "Yellow Submarine", "event_id": "145796", "event_start_utc": "2026-10-07T09:00:00Z", "features": {"away_elo": 1759.660919, "away_history_count": 286, "home_elo": 1497.898695, "home_history_count": 2}, "historical_source_observation_times_verified": false, "home_team": "Blasterbl", "inference_inputs": {"book_state": {"games_played": {"bo3:4:16486": 286, "bo3:4:23832": 2}, "inactivity_half_life_days": null, "inactivity_max_pull": null, "k": 48.0, "last_match_utc": {"bo3:4:16486": "2026-10-06T14:35:00Z", "bo3:4:23832": "2026-10-06T12:20:00Z"}, "minimum_reliable_games": null, "platt_intercept": 0.07646024717646603, "platt_slope": 0.8471774676108041, "ratings": {"bo3:4:16486": 1759.660919, "bo3:4:23832": 1497.898695}, "recency_half_life_days": null, "recency_max_boost": null, "temperature": 1.18, "thin_data_max_shrink": null, "tier_weights": null}, "code_sha256": {"esports.py": "48eab29fd660f72bcbd6f9557cca081a5e6f76c9da89c9cf36ce7181c79b1174", "features/elo_ratings.py": "8525faf022a6343c452286dbfeb17dbb043744c6bdabbe448b6b371216da439b"}, "reference_date": "2026-10-06T22:25:25.483347+00:00", "team_ids": ["bo3:4:23832", "bo3:4:16486"]}, "market_type": "moneyline", "model_version": "dota2-tiered-elo-v6", "observed_at_utc": "2026-10-06T22:25:25.483347+00:00", "probabilities": {"away": 0.640253, "home": 0.359747}, "replay_scope": "Exact serving book state, calibration, temperature, inactivity reference and thin-history adjustments; training provenance not certified.", "schema": "esports-elo-replay-v1", "snapshot_hash": "72c0f4514c8da658b54751da2293583b1dca94c0c2906e7fcb514d3472bc5bc3", "sport": "DOTA2"}</t>
         </is>
       </c>
     </row>

</xml_diff>